<commit_message>
Add 2026 JULY 18 scores
</commit_message>
<xml_diff>
--- a/data/GolfData.xlsx
+++ b/data/GolfData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Apps\GolfStats\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01380EE7-31E4-4A60-A3A4-A5267B854F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82050956-2441-492D-9E0F-7C816E073636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4BA5778-8140-4272-B97C-07E35F2520D6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4BA5778-8140-4272-B97C-07E35F2520D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Score Cards" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -1178,8 +1178,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}" name="Table1" displayName="Table1" ref="A1:W20" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
-  <autoFilter ref="A1:W20" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}" name="Table1" displayName="Table1" ref="A1:W21" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
+  <autoFilter ref="A1:W21" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}"/>
   <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{6036417A-52C2-4AF8-9A0D-25AEE607F48A}" name="Course" dataDxfId="70"/>
     <tableColumn id="2" xr3:uid="{AE08F17B-78CF-43B6-86B1-7635DA793064}" name="Date" dataDxfId="69"/>
@@ -1564,7 +1564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838B056B-02E7-4106-A28B-369A087ADF9A}">
-  <dimension ref="A1:W20"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="1" customWidth="1"/>
@@ -2992,6 +2992,77 @@
         <v>28</v>
       </c>
       <c r="W20" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C21" s="1">
+        <v>5</v>
+      </c>
+      <c r="D21" s="1">
+        <v>5</v>
+      </c>
+      <c r="E21" s="1">
+        <v>5</v>
+      </c>
+      <c r="F21" s="1">
+        <v>4</v>
+      </c>
+      <c r="G21" s="1">
+        <v>6</v>
+      </c>
+      <c r="H21" s="1">
+        <v>3</v>
+      </c>
+      <c r="I21" s="1">
+        <v>7</v>
+      </c>
+      <c r="J21" s="1">
+        <v>6</v>
+      </c>
+      <c r="K21" s="1">
+        <v>6</v>
+      </c>
+      <c r="L21" s="1">
+        <v>4</v>
+      </c>
+      <c r="M21" s="1">
+        <v>5</v>
+      </c>
+      <c r="N21" s="1">
+        <v>5</v>
+      </c>
+      <c r="O21" s="1">
+        <v>4</v>
+      </c>
+      <c r="P21" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q21" s="1">
+        <v>3</v>
+      </c>
+      <c r="R21" s="1">
+        <v>5</v>
+      </c>
+      <c r="S21" s="1">
+        <v>4</v>
+      </c>
+      <c r="T21" s="1">
+        <v>4</v>
+      </c>
+      <c r="U21" s="1">
+        <v>3</v>
+      </c>
+      <c r="V21" s="1">
+        <v>31</v>
+      </c>
+      <c r="W21" s="1">
         <v>7</v>
       </c>
     </row>

</xml_diff>